<commit_message>
Document clearance workflow redesign
</commit_message>
<xml_diff>
--- a/04.03装柜信息(1).xlsx
+++ b/04.03装柜信息(1).xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20745" windowHeight="9675"/>
+    <workbookView windowHeight="14860"/>
   </bookViews>
   <sheets>
     <sheet name="sheel" sheetId="1" r:id="rId1"/>
@@ -4365,7 +4365,7 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -5060,10 +5060,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:BP440"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
+    <col min="1" max="1" width="24.8365384615385" customWidth="1"/>
+    <col min="2" max="2" width="34.6153846153846" customWidth="1"/>
+    <col min="10" max="10" width="14.5769230769231" customWidth="1"/>
+    <col min="11" max="11" width="21.6346153846154" customWidth="1"/>
+    <col min="14" max="14" width="19.5480769230769" customWidth="1"/>
+    <col min="17" max="17" width="16.6634615384615" customWidth="1"/>
+    <col min="19" max="19" width="12.5" customWidth="1"/>
+    <col min="21" max="21" width="11.8557692307692" customWidth="1"/>
+    <col min="22" max="22" width="17.2980769230769" customWidth="1"/>
     <col min="24" max="24" width="14" customWidth="1"/>
+    <col min="25" max="25" width="12.3461538461538" customWidth="1"/>
     <col min="26" max="26" width="11.875" customWidth="1"/>
+    <col min="52" max="52" width="28.5192307692308" customWidth="1"/>
     <col min="56" max="56" width="19.375" style="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>